<commit_message>
Updated reconConfigs excel file
</commit_message>
<xml_diff>
--- a/reconConfigs.xlsx
+++ b/reconConfigs.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q217"/>
+  <dimension ref="A1:Q267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11399,6 +11399,2684 @@
       <c r="P217" t="inlineStr"/>
       <c r="Q217" t="inlineStr"/>
     </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>223</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>1203231</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>BOOKWORLD KKIA</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr"/>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="n">
+        <v>1</v>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr"/>
+      <c r="K218" t="inlineStr"/>
+      <c r="L218" t="n">
+        <v>782</v>
+      </c>
+      <c r="M218" t="n">
+        <v>0</v>
+      </c>
+      <c r="N218" s="2" t="n">
+        <v>45964.63601851852</v>
+      </c>
+      <c r="O218" s="2" t="n">
+        <v>45965.51612268519</v>
+      </c>
+      <c r="P218" t="inlineStr"/>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>224</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>1220391</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Divine Meat Empire</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr"/>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="n">
+        <v>1</v>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr"/>
+      <c r="K219" t="inlineStr"/>
+      <c r="L219" t="n">
+        <v>782</v>
+      </c>
+      <c r="M219" t="n">
+        <v>0</v>
+      </c>
+      <c r="N219" s="2" t="n">
+        <v>45964.63828703704</v>
+      </c>
+      <c r="O219" s="2" t="n">
+        <v>45965.51641203704</v>
+      </c>
+      <c r="P219" t="inlineStr"/>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>225</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>0027847</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>EPISODE INVESTMENTS</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr"/>
+      <c r="G220" t="inlineStr"/>
+      <c r="H220" t="n">
+        <v>1</v>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr"/>
+      <c r="K220" t="inlineStr"/>
+      <c r="L220" t="n">
+        <v>782</v>
+      </c>
+      <c r="M220" t="n">
+        <v>0</v>
+      </c>
+      <c r="N220" s="2" t="n">
+        <v>45964.64092592592</v>
+      </c>
+      <c r="O220" s="2" t="n">
+        <v>45965.51659722222</v>
+      </c>
+      <c r="P220" t="inlineStr"/>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>226</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>1142959</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>FAY TERRY LODGE</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr"/>
+      <c r="G221" t="inlineStr"/>
+      <c r="H221" t="n">
+        <v>1</v>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr"/>
+      <c r="K221" t="inlineStr"/>
+      <c r="L221" t="n">
+        <v>782</v>
+      </c>
+      <c r="M221" t="n">
+        <v>0</v>
+      </c>
+      <c r="N221" s="2" t="n">
+        <v>45964.64159722222</v>
+      </c>
+      <c r="O221" s="2" t="n">
+        <v>45965.51765046296</v>
+      </c>
+      <c r="P221" t="inlineStr"/>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>227</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>0047845</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>GARDEN COURT KITWE</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr"/>
+      <c r="G222" t="inlineStr"/>
+      <c r="H222" t="n">
+        <v>1</v>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr"/>
+      <c r="K222" t="inlineStr"/>
+      <c r="L222" t="n">
+        <v>782</v>
+      </c>
+      <c r="M222" t="n">
+        <v>0</v>
+      </c>
+      <c r="N222" s="2" t="n">
+        <v>45964.64217592592</v>
+      </c>
+      <c r="O222" s="2" t="n">
+        <v>45965.51793981482</v>
+      </c>
+      <c r="P222" t="inlineStr"/>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>228</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>3582</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Link Pharmacy</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr"/>
+      <c r="G223" t="inlineStr"/>
+      <c r="H223" t="n">
+        <v>1</v>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr"/>
+      <c r="K223" t="inlineStr"/>
+      <c r="L223" t="n">
+        <v>782</v>
+      </c>
+      <c r="M223" t="n">
+        <v>0</v>
+      </c>
+      <c r="N223" s="2" t="n">
+        <v>45964.64282407407</v>
+      </c>
+      <c r="O223" s="2" t="n">
+        <v>45965.51741898148</v>
+      </c>
+      <c r="P223" t="inlineStr"/>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>229</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>0000786</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Nkanza &amp; Cole Laboratories</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr"/>
+      <c r="G224" t="inlineStr"/>
+      <c r="H224" t="n">
+        <v>1</v>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr"/>
+      <c r="K224" t="inlineStr"/>
+      <c r="L224" t="n">
+        <v>782</v>
+      </c>
+      <c r="M224" t="n">
+        <v>0</v>
+      </c>
+      <c r="N224" s="2" t="n">
+        <v>45964.64416666667</v>
+      </c>
+      <c r="O224" s="2" t="n">
+        <v>45965.51721064815</v>
+      </c>
+      <c r="P224" t="inlineStr"/>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>230</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>1198043</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>PALMRIDGE PROPERTIES</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr"/>
+      <c r="G225" t="inlineStr"/>
+      <c r="H225" t="n">
+        <v>1</v>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr"/>
+      <c r="K225" t="inlineStr"/>
+      <c r="L225" t="n">
+        <v>782</v>
+      </c>
+      <c r="M225" t="n">
+        <v>0</v>
+      </c>
+      <c r="N225" s="2" t="n">
+        <v>45964.64488425926</v>
+      </c>
+      <c r="O225" s="2" t="n">
+        <v>45965.51701388889</v>
+      </c>
+      <c r="P225" t="inlineStr"/>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>231</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>1124007</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>PEBBLESTONE APARTMENTS</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr"/>
+      <c r="G226" t="inlineStr"/>
+      <c r="H226" t="n">
+        <v>1</v>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr"/>
+      <c r="K226" t="inlineStr"/>
+      <c r="L226" t="n">
+        <v>782</v>
+      </c>
+      <c r="M226" t="n">
+        <v>0</v>
+      </c>
+      <c r="N226" s="2" t="n">
+        <v>45964.64556712963</v>
+      </c>
+      <c r="O226" s="2" t="n">
+        <v>45965.51681712963</v>
+      </c>
+      <c r="P226" t="inlineStr"/>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>232</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>0041095</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>SOUTHERN CROSS MOTORS</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr"/>
+      <c r="G227" t="inlineStr"/>
+      <c r="H227" t="n">
+        <v>1</v>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr"/>
+      <c r="K227" t="inlineStr"/>
+      <c r="L227" t="n">
+        <v>782</v>
+      </c>
+      <c r="M227" t="n">
+        <v>0</v>
+      </c>
+      <c r="N227" s="2" t="n">
+        <v>45964.64604166667</v>
+      </c>
+      <c r="O227" s="2" t="n">
+        <v>45965.50716435185</v>
+      </c>
+      <c r="P227" t="inlineStr"/>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>233</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>1120450</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>VARLOSTYLES BEAUTY LTD</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr"/>
+      <c r="G228" t="inlineStr"/>
+      <c r="H228" t="n">
+        <v>1</v>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr"/>
+      <c r="K228" t="inlineStr"/>
+      <c r="L228" t="n">
+        <v>782</v>
+      </c>
+      <c r="M228" t="n">
+        <v>0</v>
+      </c>
+      <c r="N228" s="2" t="n">
+        <v>45964.64650462963</v>
+      </c>
+      <c r="O228" s="2" t="n">
+        <v>45965.51386574074</v>
+      </c>
+      <c r="P228" t="inlineStr"/>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>234</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>1222348</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Venus Center Limited</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr"/>
+      <c r="G229" t="inlineStr"/>
+      <c r="H229" t="n">
+        <v>1</v>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr"/>
+      <c r="K229" t="inlineStr"/>
+      <c r="L229" t="n">
+        <v>782</v>
+      </c>
+      <c r="M229" t="n">
+        <v>0</v>
+      </c>
+      <c r="N229" s="2" t="n">
+        <v>45964.64716435185</v>
+      </c>
+      <c r="O229" s="2" t="n">
+        <v>45965.5134375</v>
+      </c>
+      <c r="P229" t="inlineStr"/>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>235</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>0043141</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>ZAMBIA BATA - WATERFALLS</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr"/>
+      <c r="G230" t="inlineStr"/>
+      <c r="H230" t="n">
+        <v>1</v>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr"/>
+      <c r="K230" t="inlineStr"/>
+      <c r="L230" t="n">
+        <v>782</v>
+      </c>
+      <c r="M230" t="n">
+        <v>0</v>
+      </c>
+      <c r="N230" s="2" t="n">
+        <v>45964.64767361111</v>
+      </c>
+      <c r="O230" s="2" t="n">
+        <v>45965.52412037037</v>
+      </c>
+      <c r="P230" t="inlineStr"/>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>236</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>0022988</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>ZAMBIA BATA SHOE - MPIKA</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr"/>
+      <c r="G231" t="inlineStr"/>
+      <c r="H231" t="n">
+        <v>1</v>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr"/>
+      <c r="K231" t="inlineStr"/>
+      <c r="L231" t="n">
+        <v>782</v>
+      </c>
+      <c r="M231" t="n">
+        <v>0</v>
+      </c>
+      <c r="N231" s="2" t="n">
+        <v>45964.64820601852</v>
+      </c>
+      <c r="O231" s="2" t="n">
+        <v>45965.52340277778</v>
+      </c>
+      <c r="P231" t="inlineStr"/>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>237</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>1236819</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Zambia Police Chawama Traffic</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>1.25%</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" t="inlineStr"/>
+      <c r="H232" t="n">
+        <v>1</v>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr"/>
+      <c r="K232" t="inlineStr"/>
+      <c r="L232" t="n">
+        <v>782</v>
+      </c>
+      <c r="M232" t="n">
+        <v>0</v>
+      </c>
+      <c r="N232" s="2" t="n">
+        <v>45964.64868055555</v>
+      </c>
+      <c r="O232" s="2" t="n">
+        <v>45965.51133101852</v>
+      </c>
+      <c r="P232" t="inlineStr"/>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>238</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>1236884</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Zambia Police Matero Traffic</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>1.25%</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr"/>
+      <c r="G233" t="inlineStr"/>
+      <c r="H233" t="n">
+        <v>1</v>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr"/>
+      <c r="K233" t="inlineStr"/>
+      <c r="L233" t="n">
+        <v>782</v>
+      </c>
+      <c r="M233" t="n">
+        <v>0</v>
+      </c>
+      <c r="N233" s="2" t="n">
+        <v>45964.64910879629</v>
+      </c>
+      <c r="O233" s="2" t="n">
+        <v>45965.5115625</v>
+      </c>
+      <c r="P233" t="inlineStr"/>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>239</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>1236850</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Zambia Police Lusaka Division</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>1.25%</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr"/>
+      <c r="G234" t="inlineStr"/>
+      <c r="H234" t="n">
+        <v>1</v>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr"/>
+      <c r="K234" t="inlineStr"/>
+      <c r="L234" t="n">
+        <v>782</v>
+      </c>
+      <c r="M234" t="n">
+        <v>0</v>
+      </c>
+      <c r="N234" s="2" t="n">
+        <v>45964.64967592592</v>
+      </c>
+      <c r="O234" s="2" t="n">
+        <v>45965.5117824074</v>
+      </c>
+      <c r="P234" t="inlineStr"/>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>240</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>1236967</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Zambia Police SHQs</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>1.25%</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr"/>
+      <c r="G235" t="inlineStr"/>
+      <c r="H235" t="n">
+        <v>1</v>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr"/>
+      <c r="K235" t="inlineStr"/>
+      <c r="L235" t="n">
+        <v>782</v>
+      </c>
+      <c r="M235" t="n">
+        <v>0</v>
+      </c>
+      <c r="N235" s="2" t="n">
+        <v>45964.65013888889</v>
+      </c>
+      <c r="O235" s="2" t="n">
+        <v>45965.51199074074</v>
+      </c>
+      <c r="P235" t="inlineStr"/>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>241</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>1236827</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Zambia Police Traffic Control Kabwata</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>1.25%</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr"/>
+      <c r="G236" t="inlineStr"/>
+      <c r="H236" t="n">
+        <v>1</v>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr"/>
+      <c r="K236" t="inlineStr"/>
+      <c r="L236" t="n">
+        <v>782</v>
+      </c>
+      <c r="M236" t="n">
+        <v>0</v>
+      </c>
+      <c r="N236" s="2" t="n">
+        <v>45964.65762731482</v>
+      </c>
+      <c r="O236" s="2" t="n">
+        <v>45965.51521990741</v>
+      </c>
+      <c r="P236" t="inlineStr"/>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>242</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>1236983</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Zambia Police Silverest Interpol</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>1.25%</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr"/>
+      <c r="G237" t="inlineStr"/>
+      <c r="H237" t="n">
+        <v>1</v>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr"/>
+      <c r="K237" t="inlineStr"/>
+      <c r="L237" t="n">
+        <v>782</v>
+      </c>
+      <c r="M237" t="n">
+        <v>0</v>
+      </c>
+      <c r="N237" s="2" t="n">
+        <v>45964.66201388889</v>
+      </c>
+      <c r="O237" s="2" t="n">
+        <v>45965.51546296296</v>
+      </c>
+      <c r="P237" t="inlineStr"/>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>243</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>1236843</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Zambia Police Traffic Control Kafue</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>1.25%</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr"/>
+      <c r="G238" t="inlineStr"/>
+      <c r="H238" t="n">
+        <v>1</v>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr"/>
+      <c r="K238" t="inlineStr"/>
+      <c r="L238" t="n">
+        <v>782</v>
+      </c>
+      <c r="M238" t="n">
+        <v>0</v>
+      </c>
+      <c r="N238" s="2" t="n">
+        <v>45964.66251157408</v>
+      </c>
+      <c r="O238" s="2" t="n">
+        <v>45965.51587962963</v>
+      </c>
+      <c r="P238" t="inlineStr"/>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>244</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>1237080</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Zambia Police Westwood Traffic</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>1.25%</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr"/>
+      <c r="G239" t="inlineStr"/>
+      <c r="H239" t="n">
+        <v>1</v>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr"/>
+      <c r="K239" t="inlineStr"/>
+      <c r="L239" t="n">
+        <v>782</v>
+      </c>
+      <c r="M239" t="n">
+        <v>0</v>
+      </c>
+      <c r="N239" s="2" t="n">
+        <v>45964.66502314815</v>
+      </c>
+      <c r="O239" s="2" t="n">
+        <v>45965.5156712963</v>
+      </c>
+      <c r="P239" t="inlineStr"/>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>245</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>1133305</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Vinnid Enterprises Absa House</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr"/>
+      <c r="G240" t="inlineStr"/>
+      <c r="H240" t="n">
+        <v>1</v>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr"/>
+      <c r="K240" t="inlineStr"/>
+      <c r="L240" t="n">
+        <v>782</v>
+      </c>
+      <c r="M240" t="n">
+        <v>0</v>
+      </c>
+      <c r="N240" s="2" t="n">
+        <v>45964.665625</v>
+      </c>
+      <c r="O240" s="2" t="n">
+        <v>45965.51495370371</v>
+      </c>
+      <c r="P240" t="inlineStr"/>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>246</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>1258490</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr"/>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr"/>
+      <c r="G241" t="inlineStr"/>
+      <c r="H241" t="n">
+        <v>1</v>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr"/>
+      <c r="K241" t="inlineStr"/>
+      <c r="L241" t="n">
+        <v>782</v>
+      </c>
+      <c r="M241" t="n">
+        <v>0</v>
+      </c>
+      <c r="N241" s="2" t="n">
+        <v>45964.66607638889</v>
+      </c>
+      <c r="O241" s="2" t="n">
+        <v>45965.5144212963</v>
+      </c>
+      <c r="P241" t="inlineStr"/>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>247</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>1252949</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr"/>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr"/>
+      <c r="G242" t="inlineStr"/>
+      <c r="H242" t="n">
+        <v>1</v>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr"/>
+      <c r="K242" t="inlineStr"/>
+      <c r="L242" t="n">
+        <v>782</v>
+      </c>
+      <c r="M242" t="n">
+        <v>0</v>
+      </c>
+      <c r="N242" s="2" t="n">
+        <v>45964.66640046296</v>
+      </c>
+      <c r="O242" s="2" t="n">
+        <v>45965.51027777778</v>
+      </c>
+      <c r="P242" t="inlineStr"/>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>248</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>1254598</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr"/>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr"/>
+      <c r="G243" t="inlineStr"/>
+      <c r="H243" t="n">
+        <v>1</v>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr"/>
+      <c r="K243" t="inlineStr"/>
+      <c r="L243" t="n">
+        <v>782</v>
+      </c>
+      <c r="M243" t="n">
+        <v>0</v>
+      </c>
+      <c r="N243" s="2" t="n">
+        <v>45964.66744212963</v>
+      </c>
+      <c r="O243" s="2" t="n">
+        <v>45965.51054398148</v>
+      </c>
+      <c r="P243" t="inlineStr"/>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>249</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>1254614</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr"/>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr"/>
+      <c r="G244" t="inlineStr"/>
+      <c r="H244" t="n">
+        <v>1</v>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr"/>
+      <c r="K244" t="inlineStr"/>
+      <c r="L244" t="n">
+        <v>782</v>
+      </c>
+      <c r="M244" t="n">
+        <v>0</v>
+      </c>
+      <c r="N244" s="2" t="n">
+        <v>45964.66782407407</v>
+      </c>
+      <c r="O244" s="2" t="n">
+        <v>45965.50678240741</v>
+      </c>
+      <c r="P244" t="inlineStr"/>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>250</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>1254630</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr"/>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr"/>
+      <c r="G245" t="inlineStr"/>
+      <c r="H245" t="n">
+        <v>1</v>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr"/>
+      <c r="K245" t="inlineStr"/>
+      <c r="L245" t="n">
+        <v>782</v>
+      </c>
+      <c r="M245" t="n">
+        <v>0</v>
+      </c>
+      <c r="N245" s="2" t="n">
+        <v>45964.66813657407</v>
+      </c>
+      <c r="O245" s="2" t="n">
+        <v>45965.51077546296</v>
+      </c>
+      <c r="P245" t="inlineStr"/>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>251</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>1256494</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr"/>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr"/>
+      <c r="G246" t="inlineStr"/>
+      <c r="H246" t="n">
+        <v>1</v>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr"/>
+      <c r="K246" t="inlineStr"/>
+      <c r="L246" t="n">
+        <v>782</v>
+      </c>
+      <c r="M246" t="n">
+        <v>0</v>
+      </c>
+      <c r="N246" s="2" t="n">
+        <v>45964.6687962963</v>
+      </c>
+      <c r="O246" s="2" t="n">
+        <v>45965.51100694444</v>
+      </c>
+      <c r="P246" t="inlineStr"/>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>252</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>1258466</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr"/>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr"/>
+      <c r="G247" t="inlineStr"/>
+      <c r="H247" t="n">
+        <v>1</v>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr"/>
+      <c r="K247" t="inlineStr"/>
+      <c r="L247" t="n">
+        <v>782</v>
+      </c>
+      <c r="M247" t="n">
+        <v>0</v>
+      </c>
+      <c r="N247" s="2" t="n">
+        <v>45964.66902777777</v>
+      </c>
+      <c r="O247" s="2" t="n">
+        <v>45965.50997685185</v>
+      </c>
+      <c r="P247" t="inlineStr"/>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>253</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>1262609</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr"/>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr"/>
+      <c r="G248" t="inlineStr"/>
+      <c r="H248" t="n">
+        <v>1</v>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr"/>
+      <c r="K248" t="inlineStr"/>
+      <c r="L248" t="n">
+        <v>782</v>
+      </c>
+      <c r="M248" t="n">
+        <v>0</v>
+      </c>
+      <c r="N248" s="2" t="n">
+        <v>45964.66990740741</v>
+      </c>
+      <c r="O248" s="2" t="n">
+        <v>45965.50973379629</v>
+      </c>
+      <c r="P248" t="inlineStr"/>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>254</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>1265644</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr"/>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr"/>
+      <c r="G249" t="inlineStr"/>
+      <c r="H249" t="n">
+        <v>1</v>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr"/>
+      <c r="K249" t="inlineStr"/>
+      <c r="L249" t="n">
+        <v>782</v>
+      </c>
+      <c r="M249" t="n">
+        <v>0</v>
+      </c>
+      <c r="N249" s="2" t="n">
+        <v>45964.67011574074</v>
+      </c>
+      <c r="O249" s="2" t="n">
+        <v>45965.50939814815</v>
+      </c>
+      <c r="P249" t="inlineStr"/>
+      <c r="Q249" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>255</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>1266535</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr"/>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr"/>
+      <c r="G250" t="inlineStr"/>
+      <c r="H250" t="n">
+        <v>1</v>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr"/>
+      <c r="K250" t="inlineStr"/>
+      <c r="L250" t="n">
+        <v>782</v>
+      </c>
+      <c r="M250" t="n">
+        <v>0</v>
+      </c>
+      <c r="N250" s="2" t="n">
+        <v>45964.67034722222</v>
+      </c>
+      <c r="O250" s="2" t="n">
+        <v>45965.5090625</v>
+      </c>
+      <c r="P250" t="inlineStr"/>
+      <c r="Q250" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>256</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>TPS 0-5 P</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>1193564</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Oasis Oil Ngwerere</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr"/>
+      <c r="G251" t="inlineStr"/>
+      <c r="H251" t="n">
+        <v>1</v>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr"/>
+      <c r="K251" t="inlineStr"/>
+      <c r="L251" t="n">
+        <v>782</v>
+      </c>
+      <c r="M251" t="n">
+        <v>0</v>
+      </c>
+      <c r="N251" s="2" t="n">
+        <v>45964.67121527778</v>
+      </c>
+      <c r="O251" s="2" t="n">
+        <v>45965.50884259259</v>
+      </c>
+      <c r="P251" t="inlineStr"/>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>257</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>22604774</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>MAIR PHARMACY LIMITED CHALALA</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr"/>
+      <c r="G252" t="inlineStr"/>
+      <c r="H252" t="n">
+        <v>1</v>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr"/>
+      <c r="K252" t="inlineStr"/>
+      <c r="L252" t="n">
+        <v>782</v>
+      </c>
+      <c r="M252" t="n">
+        <v>0</v>
+      </c>
+      <c r="N252" s="2" t="n">
+        <v>45965.63657407407</v>
+      </c>
+      <c r="O252" s="2" t="n">
+        <v>45965.63716435185</v>
+      </c>
+      <c r="P252" t="inlineStr"/>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>258</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>22604735</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>MARCRY INVESTMENT LIMITED</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr"/>
+      <c r="G253" t="inlineStr"/>
+      <c r="H253" t="n">
+        <v>1</v>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr"/>
+      <c r="K253" t="inlineStr"/>
+      <c r="L253" t="n">
+        <v>782</v>
+      </c>
+      <c r="M253" t="n">
+        <v>0</v>
+      </c>
+      <c r="N253" s="2" t="n">
+        <v>45965.64230324074</v>
+      </c>
+      <c r="O253" s="2" t="n">
+        <v>45965.64230324074</v>
+      </c>
+      <c r="P253" t="inlineStr"/>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>259</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>22604694</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>SANKET DIAGNOSTICS ZAMBIA LIMITED</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr"/>
+      <c r="G254" t="inlineStr"/>
+      <c r="H254" t="n">
+        <v>1</v>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr"/>
+      <c r="K254" t="inlineStr"/>
+      <c r="L254" t="n">
+        <v>782</v>
+      </c>
+      <c r="M254" t="n">
+        <v>0</v>
+      </c>
+      <c r="N254" s="2" t="n">
+        <v>45965.64414351852</v>
+      </c>
+      <c r="O254" s="2" t="n">
+        <v>45965.64414351852</v>
+      </c>
+      <c r="P254" t="inlineStr"/>
+      <c r="Q254" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>260</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>22604683</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>SANKET LABORATORIES LTD-LUSAKA</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr"/>
+      <c r="G255" t="inlineStr"/>
+      <c r="H255" t="n">
+        <v>1</v>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr"/>
+      <c r="K255" t="inlineStr"/>
+      <c r="L255" t="n">
+        <v>782</v>
+      </c>
+      <c r="M255" t="n">
+        <v>0</v>
+      </c>
+      <c r="N255" s="2" t="n">
+        <v>45965.6447800926</v>
+      </c>
+      <c r="O255" s="2" t="n">
+        <v>45965.6447800926</v>
+      </c>
+      <c r="P255" t="inlineStr"/>
+      <c r="Q255" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>261</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>22604748</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>CHONGWE MUNICIPAL COUNCIL-FIELD 2</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>1.1%</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr"/>
+      <c r="G256" t="inlineStr"/>
+      <c r="H256" t="n">
+        <v>1</v>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr"/>
+      <c r="K256" t="inlineStr"/>
+      <c r="L256" t="n">
+        <v>782</v>
+      </c>
+      <c r="M256" t="n">
+        <v>0</v>
+      </c>
+      <c r="N256" s="2" t="n">
+        <v>45965.64538194444</v>
+      </c>
+      <c r="O256" s="2" t="n">
+        <v>45965.64538194444</v>
+      </c>
+      <c r="P256" t="inlineStr"/>
+      <c r="Q256" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>262</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>22604722</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>LUSAKA CITY COUNCIL</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>1.1%</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr"/>
+      <c r="G257" t="inlineStr"/>
+      <c r="H257" t="n">
+        <v>1</v>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr"/>
+      <c r="K257" t="inlineStr"/>
+      <c r="L257" t="n">
+        <v>782</v>
+      </c>
+      <c r="M257" t="n">
+        <v>0</v>
+      </c>
+      <c r="N257" s="2" t="n">
+        <v>45965.64707175926</v>
+      </c>
+      <c r="O257" s="2" t="n">
+        <v>45965.64707175926</v>
+      </c>
+      <c r="P257" t="inlineStr"/>
+      <c r="Q257" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>263</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>22604194</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>GFK TRADING LIMITED</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr"/>
+      <c r="G258" t="inlineStr"/>
+      <c r="H258" t="n">
+        <v>1</v>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr"/>
+      <c r="K258" t="inlineStr"/>
+      <c r="L258" t="n">
+        <v>782</v>
+      </c>
+      <c r="M258" t="n">
+        <v>0</v>
+      </c>
+      <c r="N258" s="2" t="n">
+        <v>45965.64878472222</v>
+      </c>
+      <c r="O258" s="2" t="n">
+        <v>45965.64878472222</v>
+      </c>
+      <c r="P258" t="inlineStr"/>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>264</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>22604712</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Oasis Chavuma.</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr"/>
+      <c r="G259" t="inlineStr"/>
+      <c r="H259" t="n">
+        <v>1</v>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr"/>
+      <c r="K259" t="inlineStr"/>
+      <c r="L259" t="n">
+        <v>782</v>
+      </c>
+      <c r="M259" t="n">
+        <v>0</v>
+      </c>
+      <c r="N259" s="2" t="n">
+        <v>45965.64931712963</v>
+      </c>
+      <c r="O259" s="2" t="n">
+        <v>45965.64931712963</v>
+      </c>
+      <c r="P259" t="inlineStr"/>
+      <c r="Q259" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>265</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>22604732</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Oasis Chongwe</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr"/>
+      <c r="G260" t="inlineStr"/>
+      <c r="H260" t="n">
+        <v>1</v>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr"/>
+      <c r="K260" t="inlineStr"/>
+      <c r="L260" t="n">
+        <v>782</v>
+      </c>
+      <c r="M260" t="n">
+        <v>0</v>
+      </c>
+      <c r="N260" s="2" t="n">
+        <v>45965.64973379629</v>
+      </c>
+      <c r="O260" s="2" t="n">
+        <v>45965.64973379629</v>
+      </c>
+      <c r="P260" t="inlineStr"/>
+      <c r="Q260" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>266</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>22604349</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>OASIS Mungwi Road</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr"/>
+      <c r="G261" t="inlineStr"/>
+      <c r="H261" t="n">
+        <v>1</v>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr"/>
+      <c r="K261" t="inlineStr"/>
+      <c r="L261" t="n">
+        <v>782</v>
+      </c>
+      <c r="M261" t="n">
+        <v>0</v>
+      </c>
+      <c r="N261" s="2" t="n">
+        <v>45965.65015046296</v>
+      </c>
+      <c r="O261" s="2" t="n">
+        <v>45965.65015046296</v>
+      </c>
+      <c r="P261" t="inlineStr"/>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>267</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>22604351</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>OASIS OIL LIMITED - NAMPUNDWE</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr"/>
+      <c r="G262" t="inlineStr"/>
+      <c r="H262" t="n">
+        <v>1</v>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr"/>
+      <c r="K262" t="inlineStr"/>
+      <c r="L262" t="n">
+        <v>782</v>
+      </c>
+      <c r="M262" t="n">
+        <v>0</v>
+      </c>
+      <c r="N262" s="2" t="n">
+        <v>45965.65052083333</v>
+      </c>
+      <c r="O262" s="2" t="n">
+        <v>45965.65052083333</v>
+      </c>
+      <c r="P262" t="inlineStr"/>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>268</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>22604762</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>OASIS OIL LIMITED-MAKENI 1</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr"/>
+      <c r="G263" t="inlineStr"/>
+      <c r="H263" t="n">
+        <v>1</v>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr"/>
+      <c r="K263" t="inlineStr"/>
+      <c r="L263" t="n">
+        <v>782</v>
+      </c>
+      <c r="M263" t="n">
+        <v>0</v>
+      </c>
+      <c r="N263" s="2" t="n">
+        <v>45965.65158564815</v>
+      </c>
+      <c r="O263" s="2" t="n">
+        <v>45965.65158564815</v>
+      </c>
+      <c r="P263" t="inlineStr"/>
+      <c r="Q263" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>269</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>22604775</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>OASIS RING RD 1</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr"/>
+      <c r="G264" t="inlineStr"/>
+      <c r="H264" t="n">
+        <v>1</v>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr"/>
+      <c r="K264" t="inlineStr"/>
+      <c r="L264" t="n">
+        <v>782</v>
+      </c>
+      <c r="M264" t="n">
+        <v>0</v>
+      </c>
+      <c r="N264" s="2" t="n">
+        <v>45965.65202546296</v>
+      </c>
+      <c r="O264" s="2" t="n">
+        <v>45965.65202546296</v>
+      </c>
+      <c r="P264" t="inlineStr"/>
+      <c r="Q264" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>270</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>UBA - ITEX</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>22604512</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>TOTAL ENERGIES LIMITED-IBEX HILL</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr"/>
+      <c r="G265" t="inlineStr"/>
+      <c r="H265" t="n">
+        <v>1</v>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr"/>
+      <c r="K265" t="inlineStr"/>
+      <c r="L265" t="n">
+        <v>782</v>
+      </c>
+      <c r="M265" t="n">
+        <v>0</v>
+      </c>
+      <c r="N265" s="2" t="n">
+        <v>45965.65243055556</v>
+      </c>
+      <c r="O265" s="2" t="n">
+        <v>45965.65243055556</v>
+      </c>
+      <c r="P265" t="inlineStr"/>
+      <c r="Q265" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>271</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Young Emerging Farmers Initiative</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr"/>
+      <c r="D266" t="inlineStr"/>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr"/>
+      <c r="G266" t="inlineStr"/>
+      <c r="H266" t="n">
+        <v>0</v>
+      </c>
+      <c r="I266" t="inlineStr"/>
+      <c r="J266" t="inlineStr"/>
+      <c r="K266" t="inlineStr"/>
+      <c r="L266" t="n">
+        <v>540</v>
+      </c>
+      <c r="M266" t="n">
+        <v>0</v>
+      </c>
+      <c r="N266" s="2" t="n">
+        <v>45971.42298611111</v>
+      </c>
+      <c r="O266" s="2" t="n">
+        <v>45971.42298611111</v>
+      </c>
+      <c r="P266" t="inlineStr"/>
+      <c r="Q266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>272</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>MOUNT ZION CHRISTIAN CENTRE</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr"/>
+      <c r="D267" t="inlineStr"/>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr"/>
+      <c r="G267" t="inlineStr"/>
+      <c r="H267" t="n">
+        <v>0</v>
+      </c>
+      <c r="I267" t="inlineStr"/>
+      <c r="J267" t="inlineStr"/>
+      <c r="K267" t="inlineStr"/>
+      <c r="L267" t="n">
+        <v>540</v>
+      </c>
+      <c r="M267" t="n">
+        <v>0</v>
+      </c>
+      <c r="N267" s="2" t="n">
+        <v>45971.42344907407</v>
+      </c>
+      <c r="O267" s="2" t="n">
+        <v>45971.42344907407</v>
+      </c>
+      <c r="P267" t="inlineStr"/>
+      <c r="Q267" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>